<commit_message>
fix(demo): draft reminders for EVERY overdue account (remove 8-cap)
- draftMode no longer caps at 8 — it drafts all overdue customers (current
  accounts are intentionally skipped; you don't remind someone who's paid).
- Remote model is only called for small batches (<=12) for token safety;
  larger sets draft instantly from compliant bilingual templates.
- Headline now reads "…for every overdue account."
- Bumped the synthetic sample to 120 customers (50 overdue) so the default
  demo feels like a real bank export.

Verified: 120-row file → 50/50 overdue drafted, 464 values protected; panel
renders all cards and scrolls.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-data/qatar-retail-portfolio.xlsx
+++ b/demo-data/qatar-retail-portfolio.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I121"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1646,9 +1646,2271 @@
         <v>45</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Khalid Al-Thani</v>
+      </c>
+      <c r="B44" t="str">
+        <v>39447475579</v>
+      </c>
+      <c r="C44" t="str">
+        <v>QA26CBQA858353618878801656442</v>
+      </c>
+      <c r="D44" t="str">
+        <v>+974 3274 8573</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F44" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G44">
+        <v>13370</v>
+      </c>
+      <c r="H44">
+        <v>7556</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Ahmed Mathew</v>
+      </c>
+      <c r="B45" t="str">
+        <v>34888544734</v>
+      </c>
+      <c r="C45" t="str">
+        <v>QA67MARK204230186480991709121</v>
+      </c>
+      <c r="D45" t="str">
+        <v>+974 6924 5205</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F45" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G45">
+        <v>51726</v>
+      </c>
+      <c r="H45">
+        <v>370970</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Hamad Al-Sulaiti</v>
+      </c>
+      <c r="B46" t="str">
+        <v>22157427644</v>
+      </c>
+      <c r="C46" t="str">
+        <v>QA75DOHB205249742627781880521</v>
+      </c>
+      <c r="D46" t="str">
+        <v>+974 5842 4234</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G46">
+        <v>37910</v>
+      </c>
+      <c r="H46">
+        <v>25981</v>
+      </c>
+      <c r="I46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Sara Khan</v>
+      </c>
+      <c r="B47" t="str">
+        <v>33478480919</v>
+      </c>
+      <c r="C47" t="str">
+        <v>QA86CBQA487345355996523256229</v>
+      </c>
+      <c r="D47" t="str">
+        <v>+974 6278 8333</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F47" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G47">
+        <v>29530</v>
+      </c>
+      <c r="H47">
+        <v>181177</v>
+      </c>
+      <c r="I47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Hamad Al-Naimi</v>
+      </c>
+      <c r="B48" t="str">
+        <v>32448969350</v>
+      </c>
+      <c r="C48" t="str">
+        <v>QA85QIBK317188720414885429504</v>
+      </c>
+      <c r="D48" t="str">
+        <v>+974 5860 3351</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F48" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G48">
+        <v>43627</v>
+      </c>
+      <c r="H48">
+        <v>711882</v>
+      </c>
+      <c r="I48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Fatima Santos</v>
+      </c>
+      <c r="B49" t="str">
+        <v>25352681374</v>
+      </c>
+      <c r="C49" t="str">
+        <v>QA57QNBA013738879681079428181</v>
+      </c>
+      <c r="D49" t="str">
+        <v>+974 5328 6157</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G49">
+        <v>47915</v>
+      </c>
+      <c r="H49">
+        <v>77585</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Mohan Santos</v>
+      </c>
+      <c r="B50" t="str">
+        <v>29356397994</v>
+      </c>
+      <c r="C50" t="str">
+        <v>QA74DOHB775497465377616574054</v>
+      </c>
+      <c r="D50" t="str">
+        <v>+974 5841 5678</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F50" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G50">
+        <v>50538</v>
+      </c>
+      <c r="H50">
+        <v>268178</v>
+      </c>
+      <c r="I50">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Fahad Khan</v>
+      </c>
+      <c r="B51" t="str">
+        <v>20520240746</v>
+      </c>
+      <c r="C51" t="str">
+        <v>QA24QIBK707768164615369176477</v>
+      </c>
+      <c r="D51" t="str">
+        <v>+974 7365 8420</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F51" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G51">
+        <v>55767</v>
+      </c>
+      <c r="H51">
+        <v>1020297</v>
+      </c>
+      <c r="I51">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Fahad Al-Thani</v>
+      </c>
+      <c r="B52" t="str">
+        <v>35874567140</v>
+      </c>
+      <c r="C52" t="str">
+        <v>QA36QIBK779140726269805266117</v>
+      </c>
+      <c r="D52" t="str">
+        <v>+974 6922 4396</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G52">
+        <v>50858</v>
+      </c>
+      <c r="H52">
+        <v>435565</v>
+      </c>
+      <c r="I52">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Mohan Santos</v>
+      </c>
+      <c r="B53" t="str">
+        <v>31089738510</v>
+      </c>
+      <c r="C53" t="str">
+        <v>QA87QNBA103211575741666753283</v>
+      </c>
+      <c r="D53" t="str">
+        <v>+974 6848 7086</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G53">
+        <v>13902</v>
+      </c>
+      <c r="H53">
+        <v>30791</v>
+      </c>
+      <c r="I53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Sara Al-Naimi</v>
+      </c>
+      <c r="B54" t="str">
+        <v>28584699024</v>
+      </c>
+      <c r="C54" t="str">
+        <v>QA72CBQA661301861716360337434</v>
+      </c>
+      <c r="D54" t="str">
+        <v>+974 3297 6791</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G54">
+        <v>48752</v>
+      </c>
+      <c r="H54">
+        <v>247744</v>
+      </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Sofia Al-Naimi</v>
+      </c>
+      <c r="B55" t="str">
+        <v>20155274476</v>
+      </c>
+      <c r="C55" t="str">
+        <v>QA63QIBK185996251473437223272</v>
+      </c>
+      <c r="D55" t="str">
+        <v>+974 3237 7573</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G55">
+        <v>39575</v>
+      </c>
+      <c r="H55">
+        <v>127108</v>
+      </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Fahad Nair</v>
+      </c>
+      <c r="B56" t="str">
+        <v>22596119779</v>
+      </c>
+      <c r="C56" t="str">
+        <v>QA49QNBA439694608108238585340</v>
+      </c>
+      <c r="D56" t="str">
+        <v>+974 5666 5807</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G56">
+        <v>23692</v>
+      </c>
+      <c r="H56">
+        <v>64449</v>
+      </c>
+      <c r="I56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Ali Al-Marri</v>
+      </c>
+      <c r="B57" t="str">
+        <v>23149922285</v>
+      </c>
+      <c r="C57" t="str">
+        <v>QA27QIBK106294384507861369984</v>
+      </c>
+      <c r="D57" t="str">
+        <v>+974 7512 3326</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F57" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G57">
+        <v>55905</v>
+      </c>
+      <c r="H57">
+        <v>208557</v>
+      </c>
+      <c r="I57">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Sara Costa</v>
+      </c>
+      <c r="B58" t="str">
+        <v>36388963434</v>
+      </c>
+      <c r="C58" t="str">
+        <v>QA90QNBA481732277043146159371</v>
+      </c>
+      <c r="D58" t="str">
+        <v>+974 7206 6965</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F58" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G58">
+        <v>42758</v>
+      </c>
+      <c r="H58">
+        <v>111879</v>
+      </c>
+      <c r="I58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>David Al-Sulaiti</v>
+      </c>
+      <c r="B59" t="str">
+        <v>36489465710</v>
+      </c>
+      <c r="C59" t="str">
+        <v>QA69DOHB944090064934947661874</v>
+      </c>
+      <c r="D59" t="str">
+        <v>+974 6418 3121</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F59" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G59">
+        <v>60364</v>
+      </c>
+      <c r="H59">
+        <v>478888</v>
+      </c>
+      <c r="I59">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Sara Al-Sulaiti</v>
+      </c>
+      <c r="B60" t="str">
+        <v>23859010888</v>
+      </c>
+      <c r="C60" t="str">
+        <v>QA77QNBA073353212245203602426</v>
+      </c>
+      <c r="D60" t="str">
+        <v>+974 5417 5189</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F60" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G60">
+        <v>18142</v>
+      </c>
+      <c r="H60">
+        <v>93823</v>
+      </c>
+      <c r="I60">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Hamad Nair</v>
+      </c>
+      <c r="B61" t="str">
+        <v>28335833813</v>
+      </c>
+      <c r="C61" t="str">
+        <v>QA76DOHB444974517632263110426</v>
+      </c>
+      <c r="D61" t="str">
+        <v>+974 3722 1027</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F61" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G61">
+        <v>61934</v>
+      </c>
+      <c r="H61">
+        <v>472919</v>
+      </c>
+      <c r="I61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>John Al-Sulaiti</v>
+      </c>
+      <c r="B62" t="str">
+        <v>22571732958</v>
+      </c>
+      <c r="C62" t="str">
+        <v>QA70QNBA650586516169784539853</v>
+      </c>
+      <c r="D62" t="str">
+        <v>+974 5785 7951</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F62" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G62">
+        <v>20906</v>
+      </c>
+      <c r="H62">
+        <v>83090</v>
+      </c>
+      <c r="I62">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Mariam Khan</v>
+      </c>
+      <c r="B63" t="str">
+        <v>36292040131</v>
+      </c>
+      <c r="C63" t="str">
+        <v>QA83CBQA346485343920285173615</v>
+      </c>
+      <c r="D63" t="str">
+        <v>+974 5460 2816</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G63">
+        <v>13274</v>
+      </c>
+      <c r="H63">
+        <v>45130</v>
+      </c>
+      <c r="I63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Omar Rahman</v>
+      </c>
+      <c r="B64" t="str">
+        <v>22943768155</v>
+      </c>
+      <c r="C64" t="str">
+        <v>QA92QNBA481754310587572275062</v>
+      </c>
+      <c r="D64" t="str">
+        <v>+974 7355 6601</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G64">
+        <v>30065</v>
+      </c>
+      <c r="H64">
+        <v>392284</v>
+      </c>
+      <c r="I64">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Hessa Pereira</v>
+      </c>
+      <c r="B65" t="str">
+        <v>22778762162</v>
+      </c>
+      <c r="C65" t="str">
+        <v>QA47QNBA002423941729096848976</v>
+      </c>
+      <c r="D65" t="str">
+        <v>+974 6141 7038</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F65" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G65">
+        <v>62886</v>
+      </c>
+      <c r="H65">
+        <v>217286</v>
+      </c>
+      <c r="I65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Priya Hussain</v>
+      </c>
+      <c r="B66" t="str">
+        <v>20855082215</v>
+      </c>
+      <c r="C66" t="str">
+        <v>QA43MARK135337971368568968893</v>
+      </c>
+      <c r="D66" t="str">
+        <v>+974 7860 8583</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F66" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G66">
+        <v>7291</v>
+      </c>
+      <c r="H66">
+        <v>121562</v>
+      </c>
+      <c r="I66">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Mohammed Al-Emadi</v>
+      </c>
+      <c r="B67" t="str">
+        <v>23367354874</v>
+      </c>
+      <c r="C67" t="str">
+        <v>QA12MARK130810762621143088305</v>
+      </c>
+      <c r="D67" t="str">
+        <v>+974 3418 8504</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G67">
+        <v>12371</v>
+      </c>
+      <c r="H67">
+        <v>26630</v>
+      </c>
+      <c r="I67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Nasser Rahman</v>
+      </c>
+      <c r="B68" t="str">
+        <v>22169238108</v>
+      </c>
+      <c r="C68" t="str">
+        <v>QA45QNBA256681470885983967556</v>
+      </c>
+      <c r="D68" t="str">
+        <v>+974 5252 5675</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G68">
+        <v>22990</v>
+      </c>
+      <c r="H68">
+        <v>36715</v>
+      </c>
+      <c r="I68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Youssef Al-Emadi</v>
+      </c>
+      <c r="B69" t="str">
+        <v>31362430754</v>
+      </c>
+      <c r="C69" t="str">
+        <v>QA13MARK953359604482177392299</v>
+      </c>
+      <c r="D69" t="str">
+        <v>+974 6522 7552</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G69">
+        <v>47693</v>
+      </c>
+      <c r="H69">
+        <v>944264</v>
+      </c>
+      <c r="I69">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Sunita Mathew</v>
+      </c>
+      <c r="B70" t="str">
+        <v>25853030961</v>
+      </c>
+      <c r="C70" t="str">
+        <v>QA13QIBK793432733777981891888</v>
+      </c>
+      <c r="D70" t="str">
+        <v>+974 5507 4646</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F70" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G70">
+        <v>50292</v>
+      </c>
+      <c r="H70">
+        <v>367852</v>
+      </c>
+      <c r="I70">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Hamad Al-Mansoori</v>
+      </c>
+      <c r="B71" t="str">
+        <v>27306255042</v>
+      </c>
+      <c r="C71" t="str">
+        <v>QA65CBQA032558856934345087847</v>
+      </c>
+      <c r="D71" t="str">
+        <v>+974 5269 5796</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F71" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G71">
+        <v>50792</v>
+      </c>
+      <c r="H71">
+        <v>169912</v>
+      </c>
+      <c r="I71">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Khalid Rahman</v>
+      </c>
+      <c r="B72" t="str">
+        <v>26965419163</v>
+      </c>
+      <c r="C72" t="str">
+        <v>QA25DOHB224521650081238271280</v>
+      </c>
+      <c r="D72" t="str">
+        <v>+974 5670 8151</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G72">
+        <v>28981</v>
+      </c>
+      <c r="H72">
+        <v>187110</v>
+      </c>
+      <c r="I72">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Priya Al-Marri</v>
+      </c>
+      <c r="B73" t="str">
+        <v>27406015435</v>
+      </c>
+      <c r="C73" t="str">
+        <v>QA96DOHB621824493962254869017</v>
+      </c>
+      <c r="D73" t="str">
+        <v>+974 5297 2303</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G73">
+        <v>61620</v>
+      </c>
+      <c r="H73">
+        <v>234194</v>
+      </c>
+      <c r="I73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Khalid Al-Thani</v>
+      </c>
+      <c r="B74" t="str">
+        <v>24221338524</v>
+      </c>
+      <c r="C74" t="str">
+        <v>QA69QNBA706278445559750638726</v>
+      </c>
+      <c r="D74" t="str">
+        <v>+974 5683 1029</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G74">
+        <v>33661</v>
+      </c>
+      <c r="H74">
+        <v>94851</v>
+      </c>
+      <c r="I74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Priya Hussain</v>
+      </c>
+      <c r="B75" t="str">
+        <v>38111167430</v>
+      </c>
+      <c r="C75" t="str">
+        <v>QA84QNBA904769758860025706748</v>
+      </c>
+      <c r="D75" t="str">
+        <v>+974 5972 5365</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F75" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G75">
+        <v>10818</v>
+      </c>
+      <c r="H75">
+        <v>105452</v>
+      </c>
+      <c r="I75">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Sunita Mathew</v>
+      </c>
+      <c r="B76" t="str">
+        <v>38723906614</v>
+      </c>
+      <c r="C76" t="str">
+        <v>QA34QIBK249242903500973899223</v>
+      </c>
+      <c r="D76" t="str">
+        <v>+974 7874 1388</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G76">
+        <v>61227</v>
+      </c>
+      <c r="H76">
+        <v>175053</v>
+      </c>
+      <c r="I76">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Omar Nair</v>
+      </c>
+      <c r="B77" t="str">
+        <v>36991643707</v>
+      </c>
+      <c r="C77" t="str">
+        <v>QA37CBQA503736305482574466451</v>
+      </c>
+      <c r="D77" t="str">
+        <v>+974 3324 9937</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F77" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G77">
+        <v>58554</v>
+      </c>
+      <c r="H77">
+        <v>278864</v>
+      </c>
+      <c r="I77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Dana Fernandes</v>
+      </c>
+      <c r="B78" t="str">
+        <v>33251821225</v>
+      </c>
+      <c r="C78" t="str">
+        <v>QA77MARK295266296098049482584</v>
+      </c>
+      <c r="D78" t="str">
+        <v>+974 7174 2090</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G78">
+        <v>19826</v>
+      </c>
+      <c r="H78">
+        <v>4103</v>
+      </c>
+      <c r="I78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Grace Fernandes</v>
+      </c>
+      <c r="B79" t="str">
+        <v>36990715675</v>
+      </c>
+      <c r="C79" t="str">
+        <v>QA20MARK629492239063422837890</v>
+      </c>
+      <c r="D79" t="str">
+        <v>+974 7486 3999</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G79">
+        <v>33004</v>
+      </c>
+      <c r="H79">
+        <v>76969</v>
+      </c>
+      <c r="I79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Fahad Rahman</v>
+      </c>
+      <c r="B80" t="str">
+        <v>29773403331</v>
+      </c>
+      <c r="C80" t="str">
+        <v>QA10MARK473783193224045812920</v>
+      </c>
+      <c r="D80" t="str">
+        <v>+974 7210 1163</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G80">
+        <v>24493</v>
+      </c>
+      <c r="H80">
+        <v>32458</v>
+      </c>
+      <c r="I80">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Rajesh Nair</v>
+      </c>
+      <c r="B81" t="str">
+        <v>21252914571</v>
+      </c>
+      <c r="C81" t="str">
+        <v>QA59MARK006667600913347625175</v>
+      </c>
+      <c r="D81" t="str">
+        <v>+974 5420 5104</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F81" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G81">
+        <v>36279</v>
+      </c>
+      <c r="H81">
+        <v>348740</v>
+      </c>
+      <c r="I81">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Mariam Hussain</v>
+      </c>
+      <c r="B82" t="str">
+        <v>27686330149</v>
+      </c>
+      <c r="C82" t="str">
+        <v>QA14CBQA369226069815708052683</v>
+      </c>
+      <c r="D82" t="str">
+        <v>+974 5222 2367</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F82" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G82">
+        <v>36488</v>
+      </c>
+      <c r="H82">
+        <v>488974</v>
+      </c>
+      <c r="I82">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Youssef Al-Thani</v>
+      </c>
+      <c r="B83" t="str">
+        <v>37933018820</v>
+      </c>
+      <c r="C83" t="str">
+        <v>QA17QIBK587956232943382799915</v>
+      </c>
+      <c r="D83" t="str">
+        <v>+974 5980 4999</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F83" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G83">
+        <v>29064</v>
+      </c>
+      <c r="H83">
+        <v>45402</v>
+      </c>
+      <c r="I83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Ahmed Al-Marri</v>
+      </c>
+      <c r="B84" t="str">
+        <v>33493655601</v>
+      </c>
+      <c r="C84" t="str">
+        <v>QA68DOHB617945302871647162548</v>
+      </c>
+      <c r="D84" t="str">
+        <v>+974 5184 7304</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F84" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G84">
+        <v>59194</v>
+      </c>
+      <c r="H84">
+        <v>485027</v>
+      </c>
+      <c r="I84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Youssef Al-Naimi</v>
+      </c>
+      <c r="B85" t="str">
+        <v>38903510995</v>
+      </c>
+      <c r="C85" t="str">
+        <v>QA76CBQA557077281003178005542</v>
+      </c>
+      <c r="D85" t="str">
+        <v>+974 3412 3681</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F85" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G85">
+        <v>54193</v>
+      </c>
+      <c r="H85">
+        <v>638270</v>
+      </c>
+      <c r="I85">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Noora Nair</v>
+      </c>
+      <c r="B86" t="str">
+        <v>36326231500</v>
+      </c>
+      <c r="C86" t="str">
+        <v>QA54DOHB385360855111742502833</v>
+      </c>
+      <c r="D86" t="str">
+        <v>+974 3144 8070</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F86" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G86">
+        <v>13598</v>
+      </c>
+      <c r="H86">
+        <v>117701</v>
+      </c>
+      <c r="I86">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Sofia Nair</v>
+      </c>
+      <c r="B87" t="str">
+        <v>29842373326</v>
+      </c>
+      <c r="C87" t="str">
+        <v>QA73MARK361198748106949449641</v>
+      </c>
+      <c r="D87" t="str">
+        <v>+974 3905 1694</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G87">
+        <v>39028</v>
+      </c>
+      <c r="H87">
+        <v>245659</v>
+      </c>
+      <c r="I87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Maha Al-Kuwari</v>
+      </c>
+      <c r="B88" t="str">
+        <v>20099309584</v>
+      </c>
+      <c r="C88" t="str">
+        <v>QA58QNBA222344313026933154024</v>
+      </c>
+      <c r="D88" t="str">
+        <v>+974 6140 9299</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G88">
+        <v>42023</v>
+      </c>
+      <c r="H88">
+        <v>35502</v>
+      </c>
+      <c r="I88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Imran Al-Thani</v>
+      </c>
+      <c r="B89" t="str">
+        <v>32150928324</v>
+      </c>
+      <c r="C89" t="str">
+        <v>QA34QNBA394100733039069102934</v>
+      </c>
+      <c r="D89" t="str">
+        <v>+974 5548 9847</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F89" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G89">
+        <v>28226</v>
+      </c>
+      <c r="H89">
+        <v>3062</v>
+      </c>
+      <c r="I89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Jassim Pereira</v>
+      </c>
+      <c r="B90" t="str">
+        <v>36302244602</v>
+      </c>
+      <c r="C90" t="str">
+        <v>QA99MARK861729895770022917964</v>
+      </c>
+      <c r="D90" t="str">
+        <v>+974 3371 5204</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G90">
+        <v>11437</v>
+      </c>
+      <c r="H90">
+        <v>43367</v>
+      </c>
+      <c r="I90">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Sara Khan</v>
+      </c>
+      <c r="B91" t="str">
+        <v>39854868174</v>
+      </c>
+      <c r="C91" t="str">
+        <v>QA10CBQA238522945703453751617</v>
+      </c>
+      <c r="D91" t="str">
+        <v>+974 5634 7019</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G91">
+        <v>41264</v>
+      </c>
+      <c r="H91">
+        <v>125228</v>
+      </c>
+      <c r="I91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Nasser Al-Thani</v>
+      </c>
+      <c r="B92" t="str">
+        <v>28088684937</v>
+      </c>
+      <c r="C92" t="str">
+        <v>QA54QIBK315035000977358391657</v>
+      </c>
+      <c r="D92" t="str">
+        <v>+974 5495 6668</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F92" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G92">
+        <v>48826</v>
+      </c>
+      <c r="H92">
+        <v>45021</v>
+      </c>
+      <c r="I92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Hamad Al-Thani</v>
+      </c>
+      <c r="B93" t="str">
+        <v>37207827945</v>
+      </c>
+      <c r="C93" t="str">
+        <v>QA37DOHB569437372149517400653</v>
+      </c>
+      <c r="D93" t="str">
+        <v>+974 7431 4770</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F93" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G93">
+        <v>37392</v>
+      </c>
+      <c r="H93">
+        <v>188236</v>
+      </c>
+      <c r="I93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Noora Al-Thani</v>
+      </c>
+      <c r="B94" t="str">
+        <v>27732155880</v>
+      </c>
+      <c r="C94" t="str">
+        <v>QA19DOHB896841484939097717740</v>
+      </c>
+      <c r="D94" t="str">
+        <v>+974 6223 4233</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F94" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G94">
+        <v>12096</v>
+      </c>
+      <c r="H94">
+        <v>177964</v>
+      </c>
+      <c r="I94">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>David Al-Emadi</v>
+      </c>
+      <c r="B95" t="str">
+        <v>39089304871</v>
+      </c>
+      <c r="C95" t="str">
+        <v>QA38CBQA026809707371564838225</v>
+      </c>
+      <c r="D95" t="str">
+        <v>+974 6553 2310</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F95" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G95">
+        <v>15619</v>
+      </c>
+      <c r="H95">
+        <v>101464</v>
+      </c>
+      <c r="I95">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Fatima Pereira</v>
+      </c>
+      <c r="B96" t="str">
+        <v>36357453026</v>
+      </c>
+      <c r="C96" t="str">
+        <v>QA28MARK842280640852599797999</v>
+      </c>
+      <c r="D96" t="str">
+        <v>+974 7266 2676</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F96" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G96">
+        <v>12865</v>
+      </c>
+      <c r="H96">
+        <v>24678</v>
+      </c>
+      <c r="I96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Maria Al-Emadi</v>
+      </c>
+      <c r="B97" t="str">
+        <v>24757706605</v>
+      </c>
+      <c r="C97" t="str">
+        <v>QA23QIBK078257800936937613517</v>
+      </c>
+      <c r="D97" t="str">
+        <v>+974 7230 8586</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F97" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G97">
+        <v>48193</v>
+      </c>
+      <c r="H97">
+        <v>360443</v>
+      </c>
+      <c r="I97">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Imran Al-Mansoori</v>
+      </c>
+      <c r="B98" t="str">
+        <v>23664547068</v>
+      </c>
+      <c r="C98" t="str">
+        <v>QA35QIBK332338001828448653641</v>
+      </c>
+      <c r="D98" t="str">
+        <v>+974 5767 1979</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F98" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G98">
+        <v>12334</v>
+      </c>
+      <c r="H98">
+        <v>4937</v>
+      </c>
+      <c r="I98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Mariam Hussain</v>
+      </c>
+      <c r="B99" t="str">
+        <v>22564280555</v>
+      </c>
+      <c r="C99" t="str">
+        <v>QA37QNBA040550856945728699070</v>
+      </c>
+      <c r="D99" t="str">
+        <v>+974 3862 7172</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F99" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G99">
+        <v>32033</v>
+      </c>
+      <c r="H99">
+        <v>34025</v>
+      </c>
+      <c r="I99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Rajesh Al-Marri</v>
+      </c>
+      <c r="B100" t="str">
+        <v>22452764133</v>
+      </c>
+      <c r="C100" t="str">
+        <v>QA75CBQA479603606840113601662</v>
+      </c>
+      <c r="D100" t="str">
+        <v>+974 6282 4056</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F100" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G100">
+        <v>62564</v>
+      </c>
+      <c r="H100">
+        <v>171945</v>
+      </c>
+      <c r="I100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Noora Al-Marri</v>
+      </c>
+      <c r="B101" t="str">
+        <v>27093750588</v>
+      </c>
+      <c r="C101" t="str">
+        <v>QA67CBQA114386188696088735085</v>
+      </c>
+      <c r="D101" t="str">
+        <v>+974 5173 4762</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F101" t="str">
+        <v>West Bay</v>
+      </c>
+      <c r="G101">
+        <v>64025</v>
+      </c>
+      <c r="H101">
+        <v>11</v>
+      </c>
+      <c r="I101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Ahmed Rahman</v>
+      </c>
+      <c r="B102" t="str">
+        <v>37784903168</v>
+      </c>
+      <c r="C102" t="str">
+        <v>QA63QIBK975963681349016690186</v>
+      </c>
+      <c r="D102" t="str">
+        <v>+974 3761 6986</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F102" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G102">
+        <v>59045</v>
+      </c>
+      <c r="H102">
+        <v>189241</v>
+      </c>
+      <c r="I102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Maria Nair</v>
+      </c>
+      <c r="B103" t="str">
+        <v>27413158397</v>
+      </c>
+      <c r="C103" t="str">
+        <v>QA50QNBA195934617784023507153</v>
+      </c>
+      <c r="D103" t="str">
+        <v>+974 3777 6833</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F103" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G103">
+        <v>13148</v>
+      </c>
+      <c r="H103">
+        <v>209253</v>
+      </c>
+      <c r="I103">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Aisha Pereira</v>
+      </c>
+      <c r="B104" t="str">
+        <v>37057368037</v>
+      </c>
+      <c r="C104" t="str">
+        <v>QA51CBQA006309990181756002427</v>
+      </c>
+      <c r="D104" t="str">
+        <v>+974 3738 8577</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F104" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G104">
+        <v>19607</v>
+      </c>
+      <c r="H104">
+        <v>47705</v>
+      </c>
+      <c r="I104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Maha Al-Mansoori</v>
+      </c>
+      <c r="B105" t="str">
+        <v>30362481557</v>
+      </c>
+      <c r="C105" t="str">
+        <v>QA23QNBA124648857616851243933</v>
+      </c>
+      <c r="D105" t="str">
+        <v>+974 7992 5091</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F105" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G105">
+        <v>36141</v>
+      </c>
+      <c r="H105">
+        <v>449980</v>
+      </c>
+      <c r="I105">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Mohan Santos</v>
+      </c>
+      <c r="B106" t="str">
+        <v>31554262549</v>
+      </c>
+      <c r="C106" t="str">
+        <v>QA60DOHB970799462140119394116</v>
+      </c>
+      <c r="D106" t="str">
+        <v>+974 6416 5347</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F106" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G106">
+        <v>57264</v>
+      </c>
+      <c r="H106">
+        <v>54151</v>
+      </c>
+      <c r="I106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Dana Al-Marri</v>
+      </c>
+      <c r="B107" t="str">
+        <v>33893375747</v>
+      </c>
+      <c r="C107" t="str">
+        <v>QA93MARK323345959710130194248</v>
+      </c>
+      <c r="D107" t="str">
+        <v>+974 7861 7895</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F107" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G107">
+        <v>41758</v>
+      </c>
+      <c r="H107">
+        <v>89712</v>
+      </c>
+      <c r="I107">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Sara Khan</v>
+      </c>
+      <c r="B108" t="str">
+        <v>28051682542</v>
+      </c>
+      <c r="C108" t="str">
+        <v>QA28DOHB623044094274594218206</v>
+      </c>
+      <c r="D108" t="str">
+        <v>+974 3695 3472</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F108" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G108">
+        <v>39314</v>
+      </c>
+      <c r="H108">
+        <v>323956</v>
+      </c>
+      <c r="I108">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Aisha Al-Thani</v>
+      </c>
+      <c r="B109" t="str">
+        <v>30068560565</v>
+      </c>
+      <c r="C109" t="str">
+        <v>QA94CBQA241049466771256713768</v>
+      </c>
+      <c r="D109" t="str">
+        <v>+974 3652 3191</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F109" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G109">
+        <v>19232</v>
+      </c>
+      <c r="H109">
+        <v>230276</v>
+      </c>
+      <c r="I109">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Mariam Fernandes</v>
+      </c>
+      <c r="B110" t="str">
+        <v>27762500842</v>
+      </c>
+      <c r="C110" t="str">
+        <v>QA12DOHB541823909151829414580</v>
+      </c>
+      <c r="D110" t="str">
+        <v>+974 6896 7417</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F110" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G110">
+        <v>11814</v>
+      </c>
+      <c r="H110">
+        <v>18273</v>
+      </c>
+      <c r="I110">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>David Fernandes</v>
+      </c>
+      <c r="B111" t="str">
+        <v>27184295562</v>
+      </c>
+      <c r="C111" t="str">
+        <v>QA79DOHB699268944389327547335</v>
+      </c>
+      <c r="D111" t="str">
+        <v>+974 7504 4537</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F111" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G111">
+        <v>46692</v>
+      </c>
+      <c r="H111">
+        <v>58714</v>
+      </c>
+      <c r="I111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Hessa Fernandes</v>
+      </c>
+      <c r="B112" t="str">
+        <v>34901734281</v>
+      </c>
+      <c r="C112" t="str">
+        <v>QA60QIBK790616346793579066714</v>
+      </c>
+      <c r="D112" t="str">
+        <v>+974 3684 2842</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="F112" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G112">
+        <v>29565</v>
+      </c>
+      <c r="H112">
+        <v>172167</v>
+      </c>
+      <c r="I112">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>David Mathew</v>
+      </c>
+      <c r="B113" t="str">
+        <v>32401590530</v>
+      </c>
+      <c r="C113" t="str">
+        <v>QA67QNBA989101541201714709152</v>
+      </c>
+      <c r="D113" t="str">
+        <v>+974 5742 1843</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F113" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G113">
+        <v>14965</v>
+      </c>
+      <c r="H113">
+        <v>50841</v>
+      </c>
+      <c r="I113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Sunita Mathew</v>
+      </c>
+      <c r="B114" t="str">
+        <v>37549840043</v>
+      </c>
+      <c r="C114" t="str">
+        <v>QA44QNBA911345106650574718950</v>
+      </c>
+      <c r="D114" t="str">
+        <v>+974 5988 7760</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F114" t="str">
+        <v>The Pearl</v>
+      </c>
+      <c r="G114">
+        <v>36332</v>
+      </c>
+      <c r="H114">
+        <v>10965</v>
+      </c>
+      <c r="I114">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Mohammed Al-Kuwari</v>
+      </c>
+      <c r="B115" t="str">
+        <v>27921062828</v>
+      </c>
+      <c r="C115" t="str">
+        <v>QA93MARK298443535350409241719</v>
+      </c>
+      <c r="D115" t="str">
+        <v>+974 5936 3199</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F115" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G115">
+        <v>11930</v>
+      </c>
+      <c r="H115">
+        <v>82291</v>
+      </c>
+      <c r="I115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Grace Al-Thani</v>
+      </c>
+      <c r="B116" t="str">
+        <v>34133455526</v>
+      </c>
+      <c r="C116" t="str">
+        <v>QA93MARK787692195098931055936</v>
+      </c>
+      <c r="D116" t="str">
+        <v>+974 3457 6531</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F116" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G116">
+        <v>16099</v>
+      </c>
+      <c r="H116">
+        <v>38395</v>
+      </c>
+      <c r="I116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Imran Mathew</v>
+      </c>
+      <c r="B117" t="str">
+        <v>29762604220</v>
+      </c>
+      <c r="C117" t="str">
+        <v>QA76DOHB704569965602445728651</v>
+      </c>
+      <c r="D117" t="str">
+        <v>+974 3223 2853</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="F117" t="str">
+        <v>Al Sadd</v>
+      </c>
+      <c r="G117">
+        <v>7802</v>
+      </c>
+      <c r="H117">
+        <v>2270</v>
+      </c>
+      <c r="I117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Sofia Al-Thani</v>
+      </c>
+      <c r="B118" t="str">
+        <v>23989721592</v>
+      </c>
+      <c r="C118" t="str">
+        <v>QA11CBQA211910295697746686265</v>
+      </c>
+      <c r="D118" t="str">
+        <v>+974 5210 9947</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Home Finance</v>
+      </c>
+      <c r="F118" t="str">
+        <v>Doha City Center</v>
+      </c>
+      <c r="G118">
+        <v>34703</v>
+      </c>
+      <c r="H118">
+        <v>563634</v>
+      </c>
+      <c r="I118">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Sofia Nair</v>
+      </c>
+      <c r="B119" t="str">
+        <v>29559380783</v>
+      </c>
+      <c r="C119" t="str">
+        <v>QA57DOHB018749145338646423286</v>
+      </c>
+      <c r="D119" t="str">
+        <v>+974 6636 7939</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F119" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G119">
+        <v>34179</v>
+      </c>
+      <c r="H119">
+        <v>98387</v>
+      </c>
+      <c r="I119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Aisha Al-Thani</v>
+      </c>
+      <c r="B120" t="str">
+        <v>23637007682</v>
+      </c>
+      <c r="C120" t="str">
+        <v>QA77MARK013282329067409869678</v>
+      </c>
+      <c r="D120" t="str">
+        <v>+974 7510 4996</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Auto Loan</v>
+      </c>
+      <c r="F120" t="str">
+        <v>Lusail</v>
+      </c>
+      <c r="G120">
+        <v>24868</v>
+      </c>
+      <c r="H120">
+        <v>49334</v>
+      </c>
+      <c r="I120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Hamad Costa</v>
+      </c>
+      <c r="B121" t="str">
+        <v>21593426372</v>
+      </c>
+      <c r="C121" t="str">
+        <v>QA12CBQA142163965322362121860</v>
+      </c>
+      <c r="D121" t="str">
+        <v>+974 5589 4060</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Salary Advance</v>
+      </c>
+      <c r="F121" t="str">
+        <v>Al Rayyan</v>
+      </c>
+      <c r="G121">
+        <v>17049</v>
+      </c>
+      <c r="H121">
+        <v>91499</v>
+      </c>
+      <c r="I121">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I121"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>